<commit_message>
armo estrictira codigo, codigo main y modulos
</commit_message>
<xml_diff>
--- a/notebooks_senales/tablas_prism_grafico.xlsx
+++ b/notebooks_senales/tablas_prism_grafico.xlsx
@@ -875,100 +875,100 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-10.3303</v>
+        <v>-10.2849</v>
       </c>
       <c r="C3" t="n">
-        <v>-10.6501</v>
+        <v>-10.5173</v>
       </c>
       <c r="D3" t="n">
-        <v>-8.942500000000001</v>
+        <v>-9.1554</v>
       </c>
       <c r="E3" t="n">
-        <v>-10.3656</v>
+        <v>-10.2096</v>
       </c>
       <c r="F3" t="n">
-        <v>-10.5361</v>
+        <v>-10.5576</v>
       </c>
       <c r="G3" t="n">
-        <v>-10.923</v>
+        <v>-10.8826</v>
       </c>
       <c r="H3" t="n">
-        <v>-10.2795</v>
+        <v>-10.156</v>
       </c>
       <c r="I3" t="n">
-        <v>-10.12</v>
+        <v>-10.1195</v>
       </c>
       <c r="J3" t="n">
-        <v>-10.3319</v>
+        <v>-10.3811</v>
       </c>
       <c r="K3" t="n">
-        <v>-10.6569</v>
+        <v>-10.5467</v>
       </c>
       <c r="M3" t="n">
-        <v>-10.6652</v>
+        <v>-10.6098</v>
       </c>
       <c r="N3" t="n">
-        <v>-11.0642</v>
+        <v>-11.0409</v>
       </c>
       <c r="O3" t="n">
-        <v>-10.6329</v>
+        <v>-10.5447</v>
       </c>
       <c r="P3" t="n">
-        <v>-10.7224</v>
+        <v>-10.7307</v>
       </c>
       <c r="Q3" t="n">
-        <v>-10.9526</v>
+        <v>-10.9357</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.2165</v>
+        <v>-11.2067</v>
       </c>
       <c r="S3" t="n">
-        <v>-10.4743</v>
+        <v>-10.4782</v>
       </c>
       <c r="T3" t="n">
-        <v>-10.7711</v>
+        <v>-10.756</v>
       </c>
       <c r="U3" t="n">
-        <v>-10.9094</v>
+        <v>-10.9013</v>
       </c>
       <c r="V3" t="n">
-        <v>-10.6503</v>
+        <v>-10.6922</v>
       </c>
       <c r="X3" t="n">
-        <v>-11.1465</v>
+        <v>-10.8636</v>
       </c>
       <c r="Y3" t="n">
-        <v>-11.6466</v>
+        <v>-11.3947</v>
       </c>
       <c r="Z3" t="n">
-        <v>-11.0953</v>
+        <v>-10.723</v>
       </c>
       <c r="AA3" t="n">
-        <v>-10.8108</v>
+        <v>-10.894</v>
       </c>
       <c r="AB3" t="n">
-        <v>-11.4849</v>
+        <v>-10.7174</v>
       </c>
       <c r="AC3" t="n">
-        <v>-11.6825</v>
+        <v>-11.4802</v>
       </c>
       <c r="AD3" t="n">
-        <v>-8.9215</v>
+        <v>-9.1692</v>
       </c>
       <c r="AE3" t="n">
-        <v>-11.0386</v>
+        <v>-10.9038</v>
       </c>
       <c r="AF3" t="n">
-        <v>-10.9748</v>
+        <v>-10.7682</v>
       </c>
       <c r="AG3" t="n">
-        <v>-10.8281</v>
+        <v>-10.8471</v>
       </c>
       <c r="AI3" t="n">
         <v>-10.9099</v>
       </c>
       <c r="AJ3" t="n">
-        <v>-11.4205</v>
+        <v>-11.4204</v>
       </c>
       <c r="AK3" t="n">
         <v>-10.9954</v>
@@ -1002,103 +1002,103 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-10.8007</v>
+        <v>-10.6995</v>
       </c>
       <c r="C4" t="n">
-        <v>-10.3442</v>
+        <v>-10.2588</v>
       </c>
       <c r="D4" t="n">
-        <v>-10.8633</v>
+        <v>-10.7926</v>
       </c>
       <c r="E4" t="n">
-        <v>-10.6539</v>
+        <v>-10.5809</v>
       </c>
       <c r="F4" t="n">
-        <v>-10.4452</v>
+        <v>-10.3374</v>
       </c>
       <c r="G4" t="n">
-        <v>-10.517</v>
+        <v>-10.4672</v>
       </c>
       <c r="H4" t="n">
-        <v>-10.4311</v>
+        <v>-10.3495</v>
       </c>
       <c r="I4" t="n">
-        <v>-10.4092</v>
+        <v>-10.2244</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.4402</v>
+        <v>-10.3907</v>
       </c>
       <c r="K4" t="n">
-        <v>-11.1386</v>
+        <v>-11.1078</v>
       </c>
       <c r="L4" t="n">
-        <v>-10.8172</v>
+        <v>-10.8117</v>
       </c>
       <c r="M4" t="n">
-        <v>-11.1341</v>
+        <v>-11.0494</v>
       </c>
       <c r="N4" t="n">
-        <v>-10.6088</v>
+        <v>-10.5629</v>
       </c>
       <c r="O4" t="n">
-        <v>-11.0517</v>
+        <v>-11.0389</v>
       </c>
       <c r="P4" t="n">
-        <v>-10.6791</v>
+        <v>-10.7288</v>
       </c>
       <c r="Q4" t="n">
-        <v>-10.6682</v>
+        <v>-10.6417</v>
       </c>
       <c r="R4" t="n">
-        <v>-10.8159</v>
+        <v>-10.7779</v>
       </c>
       <c r="S4" t="n">
-        <v>-10.7213</v>
+        <v>-10.6691</v>
       </c>
       <c r="T4" t="n">
-        <v>-10.62</v>
+        <v>-10.6254</v>
       </c>
       <c r="U4" t="n">
-        <v>-10.7544</v>
+        <v>-10.7168</v>
       </c>
       <c r="V4" t="n">
-        <v>-11.4273</v>
+        <v>-11.4282</v>
       </c>
       <c r="W4" t="n">
-        <v>-11.0106</v>
+        <v>-11.0334</v>
       </c>
       <c r="X4" t="n">
-        <v>-11.5939</v>
+        <v>-10.7009</v>
       </c>
       <c r="Y4" t="n">
-        <v>-11.058</v>
+        <v>-10.7864</v>
       </c>
       <c r="Z4" t="n">
-        <v>-11.2687</v>
+        <v>-10.9615</v>
       </c>
       <c r="AA4" t="n">
-        <v>-10.809</v>
+        <v>-10.8926</v>
       </c>
       <c r="AB4" t="n">
-        <v>-11.2723</v>
+        <v>-10.9701</v>
       </c>
       <c r="AC4" t="n">
-        <v>-11.0679</v>
+        <v>-10.7652</v>
       </c>
       <c r="AD4" t="n">
-        <v>-10.925</v>
+        <v>-10.8201</v>
       </c>
       <c r="AE4" t="n">
-        <v>-10.6461</v>
+        <v>-10.686</v>
       </c>
       <c r="AF4" t="n">
-        <v>-11.1442</v>
+        <v>-11.0026</v>
       </c>
       <c r="AG4" t="n">
-        <v>-11.7958</v>
+        <v>-11.7434</v>
       </c>
       <c r="AH4" t="n">
-        <v>-11.5752</v>
+        <v>-11.3789</v>
       </c>
       <c r="AI4" t="n">
         <v>-11.3412</v>
@@ -1604,94 +1604,94 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-10.5468</v>
+        <v>-10.5362</v>
       </c>
       <c r="C3" t="n">
-        <v>-10.5752</v>
+        <v>-10.6035</v>
       </c>
       <c r="D3" t="n">
-        <v>-9.5824</v>
+        <v>-9.7195</v>
       </c>
       <c r="E3" t="n">
-        <v>-10.6891</v>
+        <v>-10.6567</v>
       </c>
       <c r="F3" t="n">
-        <v>-10.4371</v>
+        <v>-10.4774</v>
       </c>
       <c r="G3" t="n">
-        <v>-11.0135</v>
+        <v>-10.99</v>
       </c>
       <c r="H3" t="n">
-        <v>-10.6029</v>
+        <v>-10.5814</v>
       </c>
       <c r="I3" t="n">
-        <v>-10.7665</v>
+        <v>-10.7724</v>
       </c>
       <c r="J3" t="n">
-        <v>-10.9333</v>
+        <v>-10.9518</v>
       </c>
       <c r="K3" t="n">
-        <v>-10.4555</v>
+        <v>-10.4761</v>
       </c>
       <c r="M3" t="n">
-        <v>-10.7958</v>
+        <v>-10.7753</v>
       </c>
       <c r="N3" t="n">
-        <v>-10.9042</v>
+        <v>-10.9118</v>
       </c>
       <c r="O3" t="n">
-        <v>-10.3371</v>
+        <v>-10.2926</v>
       </c>
       <c r="P3" t="n">
-        <v>-10.966</v>
+        <v>-10.9675</v>
       </c>
       <c r="Q3" t="n">
-        <v>-10.7156</v>
+        <v>-10.7296</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.2684</v>
+        <v>-11.2344</v>
       </c>
       <c r="S3" t="n">
-        <v>-10.7592</v>
+        <v>-10.7624</v>
       </c>
       <c r="T3" t="n">
-        <v>-11.1528</v>
+        <v>-11.1545</v>
       </c>
       <c r="U3" t="n">
-        <v>-11.282</v>
+        <v>-11.2829</v>
       </c>
       <c r="V3" t="n">
-        <v>-10.6546</v>
+        <v>-10.6776</v>
       </c>
       <c r="X3" t="n">
-        <v>-11.289</v>
+        <v>-11.0441</v>
       </c>
       <c r="Y3" t="n">
-        <v>-11.5786</v>
+        <v>-11.2687</v>
       </c>
       <c r="Z3" t="n">
-        <v>-10.9639</v>
+        <v>-10.6549</v>
       </c>
       <c r="AA3" t="n">
-        <v>-11.4475</v>
+        <v>-11.2728</v>
       </c>
       <c r="AB3" t="n">
-        <v>-11.4306</v>
+        <v>-11.0965</v>
       </c>
       <c r="AC3" t="n">
-        <v>-11.7286</v>
+        <v>-11.4496</v>
       </c>
       <c r="AD3" t="n">
-        <v>-9.8329</v>
+        <v>-10.0611</v>
       </c>
       <c r="AE3" t="n">
-        <v>-11.466</v>
+        <v>-11.3162</v>
       </c>
       <c r="AF3" t="n">
-        <v>-11.6234</v>
+        <v>-11.4072</v>
       </c>
       <c r="AG3" t="n">
-        <v>-11.2474</v>
+        <v>-11.0685</v>
       </c>
       <c r="AI3" t="n">
         <v>-11.0611</v>
@@ -1721,7 +1721,7 @@
         <v>-11.3967</v>
       </c>
       <c r="AR3" t="n">
-        <v>-10.8244</v>
+        <v>-10.8243</v>
       </c>
     </row>
     <row r="4">
@@ -1731,103 +1731,103 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-10.8303</v>
+        <v>-10.7254</v>
       </c>
       <c r="C4" t="n">
-        <v>-10.4034</v>
+        <v>-10.4162</v>
       </c>
       <c r="D4" t="n">
-        <v>-10.8123</v>
+        <v>-10.8338</v>
       </c>
       <c r="E4" t="n">
-        <v>-10.8972</v>
+        <v>-10.9207</v>
       </c>
       <c r="F4" t="n">
-        <v>-10.0344</v>
+        <v>-9.979799999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>-10.1815</v>
+        <v>-10.2289</v>
       </c>
       <c r="H4" t="n">
-        <v>-10.5238</v>
+        <v>-10.5457</v>
       </c>
       <c r="I4" t="n">
-        <v>-10.493</v>
+        <v>-10.4528</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.0197</v>
+        <v>-10.0683</v>
       </c>
       <c r="K4" t="n">
-        <v>-11.2478</v>
+        <v>-11.2649</v>
       </c>
       <c r="L4" t="n">
-        <v>-10.8478</v>
+        <v>-10.8707</v>
       </c>
       <c r="M4" t="n">
-        <v>-11.0567</v>
+        <v>-10.9561</v>
       </c>
       <c r="N4" t="n">
-        <v>-10.5808</v>
+        <v>-10.5832</v>
       </c>
       <c r="O4" t="n">
-        <v>-10.9971</v>
+        <v>-11.0172</v>
       </c>
       <c r="P4" t="n">
-        <v>-11.0039</v>
+        <v>-11.0427</v>
       </c>
       <c r="Q4" t="n">
-        <v>-10.3858</v>
+        <v>-10.3387</v>
       </c>
       <c r="R4" t="n">
-        <v>-10.5333</v>
+        <v>-10.5342</v>
       </c>
       <c r="S4" t="n">
-        <v>-10.8953</v>
+        <v>-10.866</v>
       </c>
       <c r="T4" t="n">
-        <v>-10.6874</v>
+        <v>-10.6776</v>
       </c>
       <c r="U4" t="n">
-        <v>-10.2973</v>
+        <v>-10.3094</v>
       </c>
       <c r="V4" t="n">
-        <v>-11.4436</v>
+        <v>-11.4524</v>
       </c>
       <c r="W4" t="n">
-        <v>-11.0629</v>
+        <v>-11.0795</v>
       </c>
       <c r="X4" t="n">
-        <v>-11.6105</v>
+        <v>-10.975</v>
       </c>
       <c r="Y4" t="n">
-        <v>-11.0547</v>
+        <v>-10.8155</v>
       </c>
       <c r="Z4" t="n">
-        <v>-11.5334</v>
+        <v>-11.2842</v>
       </c>
       <c r="AA4" t="n">
-        <v>-11.3089</v>
+        <v>-11.301</v>
       </c>
       <c r="AB4" t="n">
-        <v>-11.1286</v>
+        <v>-10.7923</v>
       </c>
       <c r="AC4" t="n">
-        <v>-10.9054</v>
+        <v>-10.4812</v>
       </c>
       <c r="AD4" t="n">
-        <v>-11.3759</v>
+        <v>-11.2099</v>
       </c>
       <c r="AE4" t="n">
-        <v>-10.9995</v>
+        <v>-10.8879</v>
       </c>
       <c r="AF4" t="n">
-        <v>-10.8279</v>
+        <v>-10.6918</v>
       </c>
       <c r="AG4" t="n">
-        <v>-11.8988</v>
+        <v>-11.7272</v>
       </c>
       <c r="AH4" t="n">
-        <v>-11.6729</v>
+        <v>-11.3697</v>
       </c>
       <c r="AI4" t="n">
         <v>-11.171</v>
@@ -1848,7 +1848,7 @@
         <v>-10.5498</v>
       </c>
       <c r="AO4" t="n">
-        <v>-10.1197</v>
+        <v>-10.1196</v>
       </c>
       <c r="AP4" t="n">
         <v>-11.0661</v>
@@ -2333,94 +2333,94 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-9.9955</v>
+        <v>-9.997299999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>-10.2975</v>
+        <v>-10.306</v>
       </c>
       <c r="D3" t="n">
-        <v>-9.6463</v>
+        <v>-9.7182</v>
       </c>
       <c r="E3" t="n">
-        <v>-10.8601</v>
+        <v>-10.8402</v>
       </c>
       <c r="F3" t="n">
-        <v>-10.52</v>
+        <v>-10.5371</v>
       </c>
       <c r="G3" t="n">
-        <v>-10.9912</v>
+        <v>-10.9283</v>
       </c>
       <c r="H3" t="n">
-        <v>-10.1604</v>
+        <v>-10.1574</v>
       </c>
       <c r="I3" t="n">
-        <v>-10.3161</v>
+        <v>-10.3341</v>
       </c>
       <c r="J3" t="n">
-        <v>-10.8613</v>
+        <v>-10.8765</v>
       </c>
       <c r="K3" t="n">
-        <v>-10.019</v>
+        <v>-10.0362</v>
       </c>
       <c r="M3" t="n">
-        <v>-10.2047</v>
+        <v>-10.1996</v>
       </c>
       <c r="N3" t="n">
-        <v>-10.5571</v>
+        <v>-10.5456</v>
       </c>
       <c r="O3" t="n">
-        <v>-10.1062</v>
+        <v>-10.0941</v>
       </c>
       <c r="P3" t="n">
-        <v>-11.0883</v>
+        <v>-11.0849</v>
       </c>
       <c r="Q3" t="n">
-        <v>-10.7899</v>
+        <v>-10.7749</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.1599</v>
+        <v>-11.1059</v>
       </c>
       <c r="S3" t="n">
-        <v>-10.3699</v>
+        <v>-10.371</v>
       </c>
       <c r="T3" t="n">
-        <v>-10.5758</v>
+        <v>-10.5738</v>
       </c>
       <c r="U3" t="n">
-        <v>-11.1331</v>
+        <v>-11.1157</v>
       </c>
       <c r="V3" t="n">
-        <v>-10.234</v>
+        <v>-10.2428</v>
       </c>
       <c r="X3" t="n">
-        <v>-10.7107</v>
+        <v>-10.4907</v>
       </c>
       <c r="Y3" t="n">
-        <v>-11.1997</v>
+        <v>-10.9063</v>
       </c>
       <c r="Z3" t="n">
-        <v>-10.7533</v>
+        <v>-10.4048</v>
       </c>
       <c r="AA3" t="n">
-        <v>-11.5578</v>
+        <v>-11.4331</v>
       </c>
       <c r="AB3" t="n">
-        <v>-11.377</v>
+        <v>-11.0936</v>
       </c>
       <c r="AC3" t="n">
-        <v>-11.6308</v>
+        <v>-11.294</v>
       </c>
       <c r="AD3" t="n">
-        <v>-10.2324</v>
+        <v>-10.3692</v>
       </c>
       <c r="AE3" t="n">
-        <v>-11.062</v>
+        <v>-10.8872</v>
       </c>
       <c r="AF3" t="n">
-        <v>-11.602</v>
+        <v>-11.3669</v>
       </c>
       <c r="AG3" t="n">
-        <v>-10.998</v>
+        <v>-10.7394</v>
       </c>
       <c r="AI3" t="n">
         <v>-10.583</v>
@@ -2447,7 +2447,7 @@
         <v>-11.0307</v>
       </c>
       <c r="AQ3" t="n">
-        <v>-11.3186</v>
+        <v>-11.3185</v>
       </c>
       <c r="AR3" t="n">
         <v>-10.3672</v>
@@ -2460,103 +2460,103 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-10.2267</v>
+        <v>-10.2186</v>
       </c>
       <c r="C4" t="n">
-        <v>-9.222099999999999</v>
+        <v>-9.2376</v>
       </c>
       <c r="D4" t="n">
-        <v>-9.7875</v>
+        <v>-9.8247</v>
       </c>
       <c r="E4" t="n">
-        <v>-10.5101</v>
+        <v>-10.522</v>
       </c>
       <c r="F4" t="n">
-        <v>-9.724399999999999</v>
+        <v>-9.708600000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>-9.8985</v>
+        <v>-9.9147</v>
       </c>
       <c r="H4" t="n">
-        <v>-10.4189</v>
+        <v>-10.409</v>
       </c>
       <c r="I4" t="n">
-        <v>-9.735099999999999</v>
+        <v>-9.753</v>
       </c>
       <c r="J4" t="n">
-        <v>-9.555099999999999</v>
+        <v>-9.5769</v>
       </c>
       <c r="K4" t="n">
-        <v>-10.1175</v>
+        <v>-10.1247</v>
       </c>
       <c r="L4" t="n">
-        <v>-10.5567</v>
+        <v>-10.6054</v>
       </c>
       <c r="M4" t="n">
-        <v>-10.4257</v>
+        <v>-10.4024</v>
       </c>
       <c r="N4" t="n">
-        <v>-9.3764</v>
+        <v>-9.3889</v>
       </c>
       <c r="O4" t="n">
-        <v>-10.0309</v>
+        <v>-10.066</v>
       </c>
       <c r="P4" t="n">
-        <v>-10.5797</v>
+        <v>-10.5933</v>
       </c>
       <c r="Q4" t="n">
-        <v>-10.0457</v>
+        <v>-10.0353</v>
       </c>
       <c r="R4" t="n">
-        <v>-10.1255</v>
+        <v>-10.1138</v>
       </c>
       <c r="S4" t="n">
-        <v>-10.6473</v>
+        <v>-10.6227</v>
       </c>
       <c r="T4" t="n">
-        <v>-9.853300000000001</v>
+        <v>-9.872400000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>-9.7158</v>
+        <v>-9.7317</v>
       </c>
       <c r="V4" t="n">
+        <v>-10.2945</v>
+      </c>
+      <c r="W4" t="n">
+        <v>-10.6961</v>
+      </c>
+      <c r="X4" t="n">
+        <v>-10.6585</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>-9.7742</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-10.7331</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-10.9809</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>-10.6956</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>-10.197</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>-11.0092</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>-10.137</v>
+      </c>
+      <c r="AF4" t="n">
         <v>-10.2912</v>
       </c>
-      <c r="W4" t="n">
-        <v>-10.6559</v>
-      </c>
-      <c r="X4" t="n">
-        <v>-11.1494</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>-9.9381</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>-10.9246</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>-10.9992</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>-10.9144</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>-10.5392</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>-11.2417</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>-10.3174</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>-10.3422</v>
-      </c>
       <c r="AG4" t="n">
-        <v>-10.8446</v>
+        <v>-10.5887</v>
       </c>
       <c r="AH4" t="n">
-        <v>-11.16</v>
+        <v>-10.8441</v>
       </c>
       <c r="AI4" t="n">
         <v>-10.5711</v>
@@ -3062,97 +3062,97 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-10.2355</v>
+        <v>-10.2237</v>
       </c>
       <c r="C3" t="n">
-        <v>-10.601</v>
+        <v>-10.6188</v>
       </c>
       <c r="D3" t="n">
-        <v>-10.1321</v>
+        <v>-10.2594</v>
       </c>
       <c r="E3" t="n">
-        <v>-10.7237</v>
+        <v>-10.7199</v>
       </c>
       <c r="F3" t="n">
-        <v>-10.752</v>
+        <v>-10.6754</v>
       </c>
       <c r="G3" t="n">
-        <v>-10.9114</v>
+        <v>-10.9157</v>
       </c>
       <c r="H3" t="n">
-        <v>-10.6908</v>
+        <v>-10.6965</v>
       </c>
       <c r="I3" t="n">
-        <v>-10.8573</v>
+        <v>-10.8037</v>
       </c>
       <c r="J3" t="n">
-        <v>-10.9898</v>
+        <v>-10.9894</v>
       </c>
       <c r="K3" t="n">
-        <v>-10.8576</v>
+        <v>-10.8487</v>
       </c>
       <c r="M3" t="n">
-        <v>-10.3915</v>
+        <v>-10.3821</v>
       </c>
       <c r="N3" t="n">
-        <v>-10.9652</v>
+        <v>-10.9789</v>
       </c>
       <c r="O3" t="n">
-        <v>-10.9478</v>
+        <v>-10.8795</v>
       </c>
       <c r="P3" t="n">
-        <v>-10.9841</v>
+        <v>-10.9427</v>
       </c>
       <c r="Q3" t="n">
-        <v>-11.0506</v>
+        <v>-10.9655</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.0881</v>
+        <v>-11.0797</v>
       </c>
       <c r="S3" t="n">
-        <v>-10.8189</v>
+        <v>-10.839</v>
       </c>
       <c r="T3" t="n">
-        <v>-10.9237</v>
+        <v>-10.8446</v>
       </c>
       <c r="U3" t="n">
-        <v>-11.2802</v>
+        <v>-11.2602</v>
       </c>
       <c r="V3" t="n">
-        <v>-11.0338</v>
+        <v>-10.9842</v>
       </c>
       <c r="X3" t="n">
-        <v>-10.8832</v>
+        <v>-10.6532</v>
       </c>
       <c r="Y3" t="n">
-        <v>-11.6079</v>
+        <v>-11.3769</v>
       </c>
       <c r="Z3" t="n">
-        <v>-11.4151</v>
+        <v>-11.0929</v>
       </c>
       <c r="AA3" t="n">
-        <v>-11.5029</v>
+        <v>-11.3325</v>
       </c>
       <c r="AB3" t="n">
-        <v>-11.6266</v>
+        <v>-11.3078</v>
       </c>
       <c r="AC3" t="n">
-        <v>-11.6725</v>
+        <v>-11.4759</v>
       </c>
       <c r="AD3" t="n">
-        <v>-10.4016</v>
+        <v>-10.5845</v>
       </c>
       <c r="AE3" t="n">
-        <v>-11.3606</v>
+        <v>-11.2261</v>
       </c>
       <c r="AF3" t="n">
-        <v>-11.6713</v>
+        <v>-11.4556</v>
       </c>
       <c r="AG3" t="n">
-        <v>-11.4984</v>
+        <v>-11.3442</v>
       </c>
       <c r="AI3" t="n">
-        <v>-10.6829</v>
+        <v>-10.6828</v>
       </c>
       <c r="AJ3" t="n">
         <v>-11.4362</v>
@@ -3189,106 +3189,106 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-11.1302</v>
+        <v>-11.0352</v>
       </c>
       <c r="C4" t="n">
-        <v>-9.7973</v>
+        <v>-9.8033</v>
       </c>
       <c r="D4" t="n">
-        <v>-11.0297</v>
+        <v>-10.9841</v>
       </c>
       <c r="E4" t="n">
-        <v>-11.1577</v>
+        <v>-11.147</v>
       </c>
       <c r="F4" t="n">
-        <v>-10.5633</v>
+        <v>-10.5454</v>
       </c>
       <c r="G4" t="n">
-        <v>-10.7127</v>
+        <v>-10.7054</v>
       </c>
       <c r="H4" t="n">
-        <v>-10.2701</v>
+        <v>-10.3002</v>
       </c>
       <c r="I4" t="n">
-        <v>-10.6229</v>
+        <v>-10.5898</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.6826</v>
+        <v>-10.6793</v>
       </c>
       <c r="K4" t="n">
-        <v>-10.9768</v>
+        <v>-10.9014</v>
       </c>
       <c r="L4" t="n">
-        <v>-10.8224</v>
+        <v>-10.85</v>
       </c>
       <c r="M4" t="n">
-        <v>-11.3102</v>
+        <v>-11.2009</v>
       </c>
       <c r="N4" t="n">
-        <v>-9.9475</v>
+        <v>-9.9352</v>
       </c>
       <c r="O4" t="n">
-        <v>-11.1753</v>
+        <v>-11.131</v>
       </c>
       <c r="P4" t="n">
-        <v>-11.1691</v>
+        <v>-11.1581</v>
       </c>
       <c r="Q4" t="n">
-        <v>-10.6736</v>
+        <v>-10.6693</v>
       </c>
       <c r="R4" t="n">
-        <v>-10.9536</v>
+        <v>-10.9443</v>
       </c>
       <c r="S4" t="n">
-        <v>-10.6988</v>
+        <v>-10.6968</v>
       </c>
       <c r="T4" t="n">
-        <v>-10.7448</v>
+        <v>-10.7544</v>
       </c>
       <c r="U4" t="n">
-        <v>-10.8827</v>
+        <v>-10.8788</v>
       </c>
       <c r="V4" t="n">
-        <v>-11.122</v>
+        <v>-11.0546</v>
       </c>
       <c r="W4" t="n">
-        <v>-10.9902</v>
+        <v>-11.0013</v>
       </c>
       <c r="X4" t="n">
-        <v>-11.7042</v>
+        <v>-11.4112</v>
       </c>
       <c r="Y4" t="n">
-        <v>-10.4258</v>
+        <v>-10.2357</v>
       </c>
       <c r="Z4" t="n">
-        <v>-11.4604</v>
+        <v>-11.1903</v>
       </c>
       <c r="AA4" t="n">
-        <v>-11.426</v>
+        <v>-11.4095</v>
       </c>
       <c r="AB4" t="n">
-        <v>-10.9381</v>
+        <v>-10.8518</v>
       </c>
       <c r="AC4" t="n">
-        <v>-11.2997</v>
+        <v>-11.0494</v>
       </c>
       <c r="AD4" t="n">
-        <v>-11.377</v>
+        <v>-11.2582</v>
       </c>
       <c r="AE4" t="n">
-        <v>-11.0626</v>
+        <v>-10.9542</v>
       </c>
       <c r="AF4" t="n">
-        <v>-11.3589</v>
+        <v>-11.2228</v>
       </c>
       <c r="AG4" t="n">
-        <v>-11.4844</v>
+        <v>-11.3535</v>
       </c>
       <c r="AH4" t="n">
-        <v>-11.6669</v>
+        <v>-11.4268</v>
       </c>
       <c r="AI4" t="n">
-        <v>-11.3641</v>
+        <v>-11.364</v>
       </c>
       <c r="AJ4" t="n">
         <v>-10.2549</v>
@@ -3306,7 +3306,7 @@
         <v>-11.1413</v>
       </c>
       <c r="AO4" t="n">
-        <v>-10.4167</v>
+        <v>-10.4166</v>
       </c>
       <c r="AP4" t="n">
         <v>-11.0553</v>

</xml_diff>